<commit_message>
Regenerate all 142 with knuckle detection fix (rake=0)
- Knuckles identified by rake=0 (covers CPS and Inactive part numbers)
- Fragment filter preserves knuckle cutlets
- All 142 assemblies regenerated, zero failures
- Master List refreshed

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Master/2110r1/2110r1 @ 0.250 IPR_cutlet_data.xlsx
+++ b/Master/2110r1/2110r1 @ 0.250 IPR_cutlet_data.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -994,239 +994,239 @@
     </row>
     <row r="28">
       <c r="A28" s="6" t="n">
-        <v>3.124</v>
+        <v>3.234</v>
       </c>
       <c r="B28" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>4.5181</v>
+        <v>4.4213</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>-0.3669</v>
+        <v>-2.031</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>0.026</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n">
-        <v>2.125</v>
+        <v>1.236</v>
       </c>
       <c r="B29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C29" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="D29" s="7" t="n">
-        <v>4.6167</v>
+        <v>4.4769</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>-0.5704</v>
+        <v>-2.4668</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>0.0225</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n">
-        <v>1.126</v>
+        <v>4.238</v>
       </c>
       <c r="B30" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>4.7007</v>
+        <v>4.4793</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>-0.7764</v>
+        <v>-2.5842</v>
       </c>
       <c r="F30" s="7" t="n">
-        <v>0.0196</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n">
-        <v>5.127</v>
+        <v>3.239</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>4.7738</v>
+        <v>4.4794</v>
       </c>
       <c r="E31" s="7" t="n">
-        <v>-0.7406</v>
+        <v>-2.7851</v>
       </c>
       <c r="F31" s="7" t="n">
-        <v>0.0171</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n">
-        <v>4.128</v>
+        <v>3.124</v>
       </c>
       <c r="B32" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>4.8356</v>
+        <v>4.5181</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>-0.9689</v>
+        <v>-0.3669</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>0.0138</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n">
-        <v>5.227</v>
+        <v>2.125</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>4.8439</v>
+        <v>4.6167</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>-0.9006</v>
+        <v>-0.5704</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>0</v>
+        <v>0.0225</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
-        <v>3.129</v>
+        <v>1.126</v>
       </c>
       <c r="B34" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="7" t="n">
-        <v>4.8798</v>
+        <v>4.7007</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>-1.1961</v>
+        <v>-0.7764</v>
       </c>
       <c r="F34" s="7" t="n">
-        <v>0.0081</v>
+        <v>0.0196</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n">
-        <v>4.228</v>
+        <v>5.127</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>4.8845</v>
+        <v>4.7738</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>-1.1198</v>
+        <v>-0.7406</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>0.0001</v>
+        <v>0.0171</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
-        <v>2.13</v>
+        <v>4.128</v>
       </c>
       <c r="B36" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C36" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D36" s="7" t="n">
-        <v>4.9135</v>
+        <v>4.8356</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>-1.4268</v>
+        <v>-0.9689</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>0.0074</v>
+        <v>0.0138</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n">
-        <v>1.131</v>
+        <v>5.227</v>
       </c>
       <c r="B37" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="7" t="n">
-        <v>4.9251</v>
+        <v>4.8439</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>-1.6005</v>
+        <v>-0.9006</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>0.0017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n">
-        <v>5.132</v>
+        <v>3.129</v>
       </c>
       <c r="B38" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="7" t="n">
-        <v>4.9342</v>
+        <v>4.8798</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>-1.5721</v>
+        <v>-1.1961</v>
       </c>
       <c r="F38" s="7" t="n">
-        <v>0.0003</v>
+        <v>0.0081</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n">
-        <v>2.135</v>
+        <v>4.228</v>
       </c>
       <c r="B39" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C39" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="D39" s="7" t="n">
-        <v>4.9356</v>
+        <v>4.8845</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>-2.1764</v>
+        <v>-1.1198</v>
       </c>
       <c r="F39" s="7" t="n">
         <v>0.0001</v>
@@ -1234,42 +1234,122 @@
     </row>
     <row r="40">
       <c r="A40" s="6" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>4.9135</v>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>-1.4268</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>0.0074</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>1.131</v>
+      </c>
+      <c r="B41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>4.9251</v>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>-1.6005</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>0.0017</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>5.132</v>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>4.9342</v>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>-1.5721</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>0.0003</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>2.135</v>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>4.9356</v>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>-2.1764</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
         <v>4.133</v>
       </c>
-      <c r="B40" s="6" t="n">
+      <c r="B44" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C40" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="7" t="n">
+      <c r="C44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="7" t="n">
         <v>4.9366</v>
       </c>
-      <c r="E40" s="7" t="n">
+      <c r="E44" s="7" t="n">
         <v>-1.7876</v>
       </c>
-      <c r="F40" s="7" t="n">
+      <c r="F44" s="7" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="42">
-      <c r="E42" s="8" t="inlineStr">
+    <row r="46">
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>Count:</t>
         </is>
       </c>
-      <c r="F42" s="9" t="n">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="E43" s="8" t="inlineStr">
+      <c r="F46" s="9" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>Total Area:</t>
         </is>
       </c>
-      <c r="F43" s="10" t="n">
-        <v>1.2242</v>
+      <c r="F47" s="10" t="n">
+        <v>1.225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>